<commit_message>
Rebuild all Word, Excel and PowerPoint outputs with the toolkit fixes
Every Word output starts its front matter on page 2 (no blank page after the cover), the
Change Management register is rebuilt with its own builder and listed in the Programme
index, and trial-migration wording is tidied in the alignment pack and the register.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Alignment/BIBS_Alignment_BRD-00_Integration_Inventory_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Alignment/BIBS_Alignment_BRD-00_Integration_Inventory_v1.0.xlsx
@@ -2591,7 +2591,7 @@
       </c>
       <c r="D31" s="12" t="inlineStr">
         <is>
-          <t>What are the 12 x 5 hours? We need extended hours for batch and month-end test cycles, weekend migration trial migrations and the dress rehearsal; MSK and ElastiCache cannot be stopped.</t>
+          <t>What are the 12 x 5 hours? We need extended hours for batch and month-end test cycles, weekend trial migrations and the dress rehearsal; MSK and ElastiCache cannot be stopped.</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>Migration trial-migration loads run here (Trial migration 3)</t>
+          <t>Trial-migration loads run here (Trial migration 3)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Platform baseline in the documentation: Valkey, Gateway API, component table
Component baseline table with licences, support horizon and the annual
review in DEPLOYMENT.md (section 7), the architecture, platform, security
and configuration documents and the programme alignment pack (rebuilt).
Redis references describing the deployment now name Valkey; the edge is
described with the Gateway API and the mapping of the former Ingress rules.
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/Alignment/BIBS_Alignment_BRD-00_Integration_Inventory_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/Alignment/BIBS_Alignment_BRD-00_Integration_Inventory_v1.0.xlsx
@@ -7229,17 +7229,17 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Redis 7 with cluster mode disabled (one shard, primary + replica, TLS, AUTH); the cache clear uses SCAN and the job lock uses scripts on single keys</t>
+          <t>Valkey 8 (BSD-3-Clause, same protocol as Redis; Amazon ElastiCache for Valkey) with cluster mode disabled (one shard, primary + replica, TLS, AUTH); the cache clear uses SCAN and the job lock uses scripts on single keys</t>
         </is>
       </c>
       <c r="D9" s="25" t="inlineStr">
         <is>
-          <t>Mismatch (wording)</t>
+          <t>Mismatch (engine, wording)</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>IER: cluster mode disabled, Multi-AZ replica. A change in BIBS only if cluster mode enabled is imposed</t>
+          <t>IER: ElastiCache for Valkey 8 in place of Redis 7.x (client decision of 08-Oct-2026: Redis 7.4 and later are no longer under the BSD licence); cluster mode disabled, Multi-AZ replica. A change in BIBS only if cluster mode enabled is imposed</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -7261,17 +7261,17 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>MSK Kafka 3.6+ with SASL/SCRAM + TLS, 9 topics plus dead-letter topics, transactional outbox; no EventBridge, no schema registry</t>
+          <t>MSK Kafka 3.9 (KRaft) with SASL/SCRAM + TLS, 9 topics plus dead-letter topics, transactional outbox; no EventBridge, no schema registry</t>
         </is>
       </c>
       <c r="D10" s="25" t="inlineStr">
         <is>
-          <t>Aligned (MSK); Mismatch (EventBridge, 80 topics)</t>
+          <t>Aligned (MSK); Mismatch (version, EventBridge, 80 topics)</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>IER: 3 brokers kafka.m5.large class, 9 topics x 3 partitions; DEV / SIT with 2 brokers need a replication factor of 2</t>
+          <t>IER: Kafka 3.9 (KRaft), 3 brokers kafka.m5.large class, 9 topics x 3 partitions; DEV / SIT with 2 brokers need a replication factor of 2</t>
         </is>
       </c>
       <c r="F10" s="12" t="inlineStr">
@@ -7325,17 +7325,17 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Kubernetes Ingress to the nginx frontend, API calls proxied to the backend; JWT issued by BIBS; login rate limit in the application</t>
+          <t>Kubernetes Gateway API: Route 53 + AWS WAF + internal ALB (AWS Load Balancer Controller) for users, Apigee X for the system APIs; HTTPS to the pods; JWT issued by BIBS; login rate limit in the application</t>
         </is>
       </c>
       <c r="D12" s="25" t="inlineStr">
         <is>
-          <t>Gap</t>
+          <t>Mismatch</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>Agree one edge: Route 53 + WAF + ALB (AWS Load Balancer Controller) or ingress-nginx; Apigee only if BDO mandates it for internal APIs</t>
+          <t>IER: a Gateway API controller in place of ingress-nginx (retired by the Kubernetes project in March 2026): the AWS Load Balancer Controller, or Envoy Gateway where an environment needs it; no CloudFront, no Istio</t>
         </is>
       </c>
       <c r="F12" s="12" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>Two pods to test the Redis job lock and cache eviction across pods</t>
+          <t>Two pods to test the Valkey job lock and cache eviction across pods</t>
         </is>
       </c>
     </row>

</xml_diff>